<commit_message>
Edited Research section. Completed first draft of Feasibility section for Zeis and Ibidi solutions.
</commit_message>
<xml_diff>
--- a/Spec_Comparison.xlsx
+++ b/Spec_Comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/klpjoa002_myuct_ac_za/Documents/Vac Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="11_D0A7759AB83DD45F29185DC745A6824D86BD80F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9227CB3-E22D-4549-B143-3ECA3193A3CB}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="11_D0A7759AB83DD45F29185DC745A6824D86BD80F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{652AE926-3577-4C87-9E00-37D68790E725}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Specification Comparison" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="166">
   <si>
     <t>Pecon Incubator (Zeis)</t>
   </si>
@@ -554,6 +554,27 @@
     <t>Must handle sterlisation solutions including:
 Bleach
 70% ethenol</t>
+  </si>
+  <si>
+    <t>Ambient temperature sensor for better control</t>
+  </si>
+  <si>
+    <t>Sample feedback mode allows for better sample temp control</t>
+  </si>
+  <si>
+    <t>Allows for temperature cycling profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H301-K-FRAME </t>
+  </si>
+  <si>
+    <t>Supports multiple lids for various experimental set ups</t>
+  </si>
+  <si>
+    <t>supports multiple sample holder mounts for various culture vessels</t>
+  </si>
+  <si>
+    <t>supports perfusion and microfluidic experiments</t>
   </si>
 </sst>
 </file>
@@ -1090,9 +1111,9 @@
   <dimension ref="A1:K68"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.140625" customWidth="1"/>
-    <col min="3" max="3" width="55.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="58.140625" customWidth="1"/>
     <col min="5" max="5" width="44.5703125" customWidth="1"/>
     <col min="6" max="6" width="55.140625" customWidth="1"/>
@@ -1949,7 +1970,9 @@
       <c r="C59" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="D59" s="40"/>
+      <c r="D59" s="39" t="s">
+        <v>162</v>
+      </c>
       <c r="E59" s="40"/>
       <c r="F59" s="40"/>
       <c r="G59" s="41" t="s">
@@ -2079,8 +2102,12 @@
         <v>33</v>
       </c>
       <c r="B66" s="11"/>
-      <c r="C66" s="40"/>
-      <c r="D66" s="40"/>
+      <c r="C66" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="D66" s="40" t="s">
+        <v>163</v>
+      </c>
       <c r="E66" s="40"/>
       <c r="F66" s="40"/>
       <c r="G66" s="4" t="s">
@@ -2093,8 +2120,12 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B67" s="11"/>
-      <c r="C67" s="40"/>
-      <c r="D67" s="40"/>
+      <c r="C67" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="D67" s="40" t="s">
+        <v>164</v>
+      </c>
       <c r="E67" s="40"/>
       <c r="F67" s="40"/>
       <c r="G67" s="4" t="s">
@@ -2107,8 +2138,12 @@
     </row>
     <row r="68" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B68" s="12"/>
-      <c r="C68" s="48"/>
-      <c r="D68" s="48"/>
+      <c r="C68" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="D68" s="48" t="s">
+        <v>165</v>
+      </c>
       <c r="E68" s="48"/>
       <c r="F68" s="48"/>
       <c r="G68" s="49"/>
@@ -2300,25 +2335,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b62a2e4-f890-4533-8a96-82be7aac4a0e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D599040ADD34C343BD6FFA9EC6676CE1" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="25d50f6ed98020584f5ffbb6cea6e855">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3b62a2e4-f890-4533-8a96-82be7aac4a0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d255d492e7d8576d3af75b08059ed773" ns2:_="">
     <xsd:import namespace="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
@@ -2496,25 +2512,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75788D79-1782-45FB-AEA2-770EDC662B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{814CF905-6104-4663-98BD-FF8C89CBBDA8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b62a2e4-f890-4533-8a96-82be7aac4a0e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF657B23-6789-406F-ABCA-58A003137FA5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2530,4 +2547,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{814CF905-6104-4663-98BD-FF8C89CBBDA8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75788D79-1782-45FB-AEA2-770EDC662B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Completed first draft of specs section, design v1. worked on presentation
</commit_message>
<xml_diff>
--- a/Spec_Comparison.xlsx
+++ b/Spec_Comparison.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/klpjoa002_myuct_ac_za/Documents/Vac Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="11_D0A7759AB83DD45F29185DC745A6824D86BD80F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{652AE926-3577-4C87-9E00-37D68790E725}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="11_D0A7759AB83DD45F29185DC745A6824D86BD80F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83C28699-C8C3-47FD-A9FD-7C35E7AE6C65}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Specification Comparison" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="165">
   <si>
     <t>Pecon Incubator (Zeis)</t>
   </si>
@@ -447,13 +447,7 @@
     <t>0.5% to 20%</t>
   </si>
   <si>
-    <t>20% to 99%</t>
-  </si>
-  <si>
     <t>±0.1% vol</t>
-  </si>
-  <si>
-    <t>±5%</t>
   </si>
   <si>
     <t xml:space="preserve">±0.2°C </t>
@@ -575,6 +569,9 @@
   </si>
   <si>
     <t>supports perfusion and microfluidic experiments</t>
+  </si>
+  <si>
+    <t>90% to 99%</t>
   </si>
 </sst>
 </file>
@@ -1125,10 +1122,10 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C1" s="37" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D1" s="38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -1214,7 +1211,7 @@
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
@@ -1955,7 +1952,7 @@
     <row r="57" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B58" s="43" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
@@ -1968,21 +1965,21 @@
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B59" s="11"/>
       <c r="C59" s="39" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D59" s="39" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E59" s="40"/>
       <c r="F59" s="40"/>
       <c r="G59" s="41" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H59" s="41" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I59" s="44" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
@@ -1991,19 +1988,19 @@
       </c>
       <c r="B60" s="11"/>
       <c r="C60" s="40" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D60" s="40"/>
       <c r="E60" s="40"/>
       <c r="F60" s="40"/>
       <c r="G60" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="I60" s="45" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
@@ -2012,19 +2009,19 @@
       </c>
       <c r="B61" s="11"/>
       <c r="C61" s="40" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D61" s="40"/>
       <c r="E61" s="40"/>
       <c r="F61" s="40"/>
       <c r="G61" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I61" s="46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
@@ -2033,19 +2030,19 @@
       </c>
       <c r="B62" s="11"/>
       <c r="C62" s="40" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D62" s="40"/>
       <c r="E62" s="40"/>
       <c r="F62" s="40"/>
       <c r="G62" s="42" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H62" s="42" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I62" s="47" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
@@ -2067,16 +2064,16 @@
       </c>
       <c r="B64" s="11"/>
       <c r="C64" s="40" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D64" s="40"/>
       <c r="E64" s="40"/>
       <c r="F64" s="40"/>
       <c r="G64" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I64" s="46"/>
     </row>
@@ -2090,10 +2087,10 @@
       <c r="E65" s="40"/>
       <c r="F65" s="40"/>
       <c r="G65" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I65" s="46"/>
     </row>
@@ -2103,46 +2100,46 @@
       </c>
       <c r="B66" s="11"/>
       <c r="C66" s="40" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D66" s="40" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E66" s="40"/>
       <c r="F66" s="40"/>
       <c r="G66" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I66" s="46"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B67" s="11"/>
       <c r="C67" s="40" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D67" s="40" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E67" s="40"/>
       <c r="F67" s="40"/>
       <c r="G67" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I67" s="46"/>
     </row>
     <row r="68" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B68" s="12"/>
       <c r="C68" s="48" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D68" s="48" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E68" s="48"/>
       <c r="F68" s="48"/>
@@ -2200,7 +2197,7 @@
         <v>88</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -2219,7 +2216,7 @@
         <v>123</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>124</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -2229,19 +2226,17 @@
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>126</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="H4" s="4"/>
       <c r="K4" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -2286,7 +2281,7 @@
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -2297,10 +2292,10 @@
         <v>33</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>131</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="4"/>
@@ -2309,10 +2304,10 @@
     </row>
     <row r="10" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="C10" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D10" s="51" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="4"/>
@@ -2321,7 +2316,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C11" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -2335,6 +2330,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b62a2e4-f890-4533-8a96-82be7aac4a0e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D599040ADD34C343BD6FFA9EC6676CE1" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="25d50f6ed98020584f5ffbb6cea6e855">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3b62a2e4-f890-4533-8a96-82be7aac4a0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d255d492e7d8576d3af75b08059ed773" ns2:_="">
     <xsd:import namespace="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
@@ -2512,26 +2526,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75788D79-1782-45FB-AEA2-770EDC662B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b62a2e4-f890-4533-8a96-82be7aac4a0e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{814CF905-6104-4663-98BD-FF8C89CBBDA8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF657B23-6789-406F-ABCA-58A003137FA5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2547,22 +2560,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{814CF905-6104-4663-98BD-FF8C89CBBDA8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75788D79-1782-45FB-AEA2-770EDC662B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3b62a2e4-f890-4533-8a96-82be7aac4a0e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>